<commit_message>
creates script to add new data for update, updates project and metadata tables
</commit_message>
<xml_diff>
--- a/create_xml_R/data-raw/metadata/genetic_identification_metadata.xlsx
+++ b/create_xml_R/data-raw/metadata/genetic_identification_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/JPE/jpe-genetics-edi/create_xml_R/data-raw/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C72F9A5-7A36-E447-B9AF-602DA1CC0597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A53898-9212-5A42-874F-7B15D0E6C9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1340" yWindow="-18880" windowWidth="30240" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -207,9 +207,6 @@
     <t>2022-01-10 09:30:00</t>
   </si>
   <si>
-    <t>2025-05-11 12:35:00</t>
-  </si>
-  <si>
     <t>Unique identifier of the sample processed. Composed of location code, season, sample event, sample bin (size class), and sample number separated by an underscore.</t>
   </si>
   <si>
@@ -265,6 +262,9 @@
   </si>
   <si>
     <t>genetic_identification_data</t>
+  </si>
+  <si>
+    <t>2026-05-08 09:58:00</t>
   </si>
 </sst>
 </file>
@@ -649,13 +649,13 @@
         <v>24</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>14</v>
@@ -693,7 +693,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
@@ -710,7 +710,7 @@
         <v>55</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
@@ -737,7 +737,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>18</v>
@@ -755,7 +755,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="5"/>
       <c r="L4" s="6">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="M4" s="6">
         <v>176</v>
@@ -785,7 +785,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>14</v>
@@ -817,13 +817,13 @@
         <v>28</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>14</v>
@@ -861,7 +861,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>14</v>
@@ -893,13 +893,13 @@
         <v>30</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>14</v>
@@ -937,7 +937,7 @@
         <v>13</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>14</v>
@@ -975,7 +975,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>14</v>
@@ -1013,7 +1013,7 @@
         <v>13</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>14</v>
@@ -1045,13 +1045,13 @@
         <v>34</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>18</v>
@@ -1093,13 +1093,13 @@
         <v>35</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>18</v>
@@ -1141,13 +1141,13 @@
         <v>36</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>18</v>
@@ -1186,16 +1186,16 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>18</v>
@@ -1237,13 +1237,13 @@
         <v>37</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>14</v>
@@ -1275,13 +1275,13 @@
         <v>38</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>18</v>
@@ -1323,13 +1323,13 @@
         <v>39</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>18</v>
@@ -1371,13 +1371,13 @@
         <v>40</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>18</v>
@@ -1419,13 +1419,13 @@
         <v>41</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>18</v>
@@ -1467,13 +1467,13 @@
         <v>42</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>18</v>
@@ -1515,13 +1515,13 @@
         <v>43</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>18</v>
@@ -1563,13 +1563,13 @@
         <v>44</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>18</v>
@@ -1611,13 +1611,13 @@
         <v>45</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>18</v>
@@ -1659,13 +1659,13 @@
         <v>46</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
tackles specific edge cases identified by Sean in the S26 updates and updates metadata to match
</commit_message>
<xml_diff>
--- a/create_xml_R/data-raw/metadata/genetic_identification_metadata.xlsx
+++ b/create_xml_R/data-raw/metadata/genetic_identification_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/JPE/jpe-genetics-edi/create_xml_R/data-raw/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A53898-9212-5A42-874F-7B15D0E6C9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A484604F-2B0B-FC4C-A6EB-D666110FE5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -755,7 +755,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="5"/>
       <c r="L4" s="6">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="M4" s="6">
         <v>176</v>

</xml_diff>